<commit_message>
Remove obsolete file and update workspace configuration
- Deleted the "Bez názvu.base" file as it was no longer needed.
- Updated the workspace configuration to reflect changes in recently opened files, ensuring a more relevant and streamlined navigation experience.
</commit_message>
<xml_diff>
--- a/00_Podklady/NUKIB_Matice_MI.xlsx
+++ b/00_Podklady/NUKIB_Matice_MI.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liftrock.sharepoint.com/sites/BIMServices/Sdilene dokumenty/General/01_Zakázky/ZAK_2023_060 ŘSD Plzeň CDE koordinátor/knowledge_base/00_Podklady/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="292" documentId="8_{DD0C42CC-F2B3-4F2E-A2B2-34D2DCF07CE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C9D0232-1548-4954-BFB9-09B5D4490703}"/>
+  <xr:revisionPtr revIDLastSave="294" documentId="8_{DD0C42CC-F2B3-4F2E-A2B2-34D2DCF07CE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E989DD8-FAA2-4644-B28E-FAD9DBB570B6}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32430" yWindow="1350" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Matice přiřazení mgmt inf" sheetId="1" r:id="rId1"/>
@@ -3397,8 +3397,9 @@
   <cols>
     <col min="1" max="1" width="6.6640625" style="8" customWidth="1"/>
     <col min="2" max="2" width="70.6640625" style="2" customWidth="1"/>
-    <col min="3" max="4" width="31.109375" style="31" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="31.44140625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="31.109375" style="31" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="22" style="31" customWidth="1"/>
+    <col min="5" max="5" width="48.21875" style="3" customWidth="1"/>
     <col min="6" max="6" width="3.44140625" style="57" customWidth="1"/>
     <col min="7" max="7" width="3.6640625" style="18" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="3.109375" style="18" customWidth="1"/>
@@ -3595,7 +3596,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="162" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" ht="160.80000000000001" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>4</v>
       </c>
@@ -3648,7 +3649,7 @@
         <v>796</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" ht="24" x14ac:dyDescent="0.25">
       <c r="A6" s="37" t="s">
         <v>16</v>
       </c>
@@ -4318,7 +4319,7 @@
       <c r="N27" s="63"/>
       <c r="O27" s="66"/>
     </row>
-    <row r="28" spans="1:16" ht="34.200000000000003" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" ht="24" x14ac:dyDescent="0.25">
       <c r="A28" s="16" t="s">
         <v>110</v>
       </c>
@@ -4777,7 +4778,7 @@
       <c r="N43" s="63"/>
       <c r="O43" s="63"/>
     </row>
-    <row r="44" spans="1:17" ht="36" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:17" ht="24" x14ac:dyDescent="0.25">
       <c r="A44" s="56" t="s">
         <v>164</v>
       </c>
@@ -7267,7 +7268,7 @@
       <c r="N122" s="63"/>
       <c r="O122" s="66"/>
     </row>
-    <row r="123" spans="1:16" ht="22.8" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A123" s="9" t="s">
         <v>496</v>
       </c>
@@ -7978,7 +7979,7 @@
       <c r="N144" s="63"/>
       <c r="O144" s="65"/>
     </row>
-    <row r="145" spans="1:15" ht="22.8" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A145" s="9" t="s">
         <v>571</v>
       </c>
@@ -8015,7 +8016,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="146" spans="1:15" ht="22.8" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A146" s="7" t="s">
         <v>574</v>
       </c>
@@ -8159,7 +8160,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="150" spans="1:15" ht="22.8" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A150" s="9" t="s">
         <v>589</v>
       </c>
@@ -9017,7 +9018,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="174" spans="1:15" ht="22.8" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A174" s="9" t="s">
         <v>690</v>
       </c>
@@ -9707,36 +9708,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="26351040-a7a6-4c2d-a8c5-8e82097712a6" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="48b746f1-b314-4eb1-99d1-d36e21f31bc3">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <typ xmlns="48b746f1-b314-4eb1-99d1-d36e21f31bc3" xsi:nil="true"/>
-    <_x010d__x00ed_slo xmlns="48b746f1-b314-4eb1-99d1-d36e21f31bc3" xsi:nil="true"/>
-    <Pov_x011b__x0159_en_x00fd_ xmlns="48b746f1-b314-4eb1-99d1-d36e21f31bc3">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Pov_x011b__x0159_en_x00fd_>
-    <Status xmlns="48b746f1-b314-4eb1-99d1-d36e21f31bc3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100CB585F688DEB1347A3B5B5B8C00EFC19" ma:contentTypeVersion="23" ma:contentTypeDescription="Vytvoří nový dokument" ma:contentTypeScope="" ma:versionID="948492b1ee3f456b1d5a5e92045a9601">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="48b746f1-b314-4eb1-99d1-d36e21f31bc3" xmlns:ns3="26351040-a7a6-4c2d-a8c5-8e82097712a6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="421727d7026b2581477b2034ccb524ed" ns2:_="" ns3:_="">
     <xsd:import namespace="48b746f1-b314-4eb1-99d1-d36e21f31bc3"/>
@@ -10047,7 +10018,64 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="26351040-a7a6-4c2d-a8c5-8e82097712a6" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="48b746f1-b314-4eb1-99d1-d36e21f31bc3">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <typ xmlns="48b746f1-b314-4eb1-99d1-d36e21f31bc3" xsi:nil="true"/>
+    <_x010d__x00ed_slo xmlns="48b746f1-b314-4eb1-99d1-d36e21f31bc3" xsi:nil="true"/>
+    <Pov_x011b__x0159_en_x00fd_ xmlns="48b746f1-b314-4eb1-99d1-d36e21f31bc3">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Pov_x011b__x0159_en_x00fd_>
+    <Status xmlns="48b746f1-b314-4eb1-99d1-d36e21f31bc3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A4B1CCE-F77F-4A2E-AE94-1E46B0CEEBE6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="48b746f1-b314-4eb1-99d1-d36e21f31bc3"/>
+    <ds:schemaRef ds:uri="26351040-a7a6-4c2d-a8c5-8e82097712a6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{53D638CD-A2A0-4241-87A1-C96B93D657AA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{16169D50-B6E2-44F9-8C13-65D6DDAC5B76}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
@@ -10064,31 +10092,4 @@
     <ds:schemaRef ds:uri="48b746f1-b314-4eb1-99d1-d36e21f31bc3"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{53D638CD-A2A0-4241-87A1-C96B93D657AA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A4B1CCE-F77F-4A2E-AE94-1E46B0CEEBE6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="48b746f1-b314-4eb1-99d1-d36e21f31bc3"/>
-    <ds:schemaRef ds:uri="26351040-a7a6-4c2d-a8c5-8e82097712a6"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>